<commit_message>
Replaced the static creation of LinkedDataTerms by a function that reads a json file.
</commit_message>
<xml_diff>
--- a/src/test/resources/test-noproblems.xlsx
+++ b/src/test/resources/test-noproblems.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\mephistophilus\MyGitRepositories\ears3\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E04F5179-580A-410B-B3EF-EB612D17E1D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D166BD9-D622-4E8D-BFA4-4C162B443555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="332" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3075" yWindow="3075" windowWidth="21600" windowHeight="11295" tabRatio="332" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24299,8 +24299,12 @@
         <v>78</v>
       </c>
       <c r="L23" s="37"/>
-      <c r="M23" s="37"/>
-      <c r="N23" s="37"/>
+      <c r="M23" s="37">
+        <v>16</v>
+      </c>
+      <c r="N23" s="37">
+        <v>4</v>
+      </c>
       <c r="O23" s="37"/>
       <c r="P23" s="37"/>
       <c r="Q23" s="37"/>

</xml_diff>